<commit_message>
feat: add KALM Signature Oversized Tee draft
</commit_message>
<xml_diff>
--- a/reports/KALM-ODO-PILOT/KALM-ODO-UNIT-ECONOMICS.xlsx
+++ b/reports/KALM-ODO-PILOT/KALM-ODO-UNIT-ECONOMICS.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rd0f8c9e748174312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="Ra5e0af99def147a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity scenarios" sheetId="3" r:id="Rf190be49876e48b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODO sensitivity" sheetId="4" r:id="Rddda92d4e76d4b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="Rbef4158669b44c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R1c3993f033824882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R04b0d82e10584bb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity scenarios" sheetId="3" r:id="R664b947ac70f40ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODO sensitivity" sheetId="4" r:id="R2887ae4e08654c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="Rc2238fdabf06441b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -337,38 +337,59 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>KALM COLLECTIVE — ODO PREMIUM EMBROIDERED T-SHIRT UNIT ECONOMICS</x:v>
+        <x:v>KALM COLLECTIVE — KALM SIGNATURE OVERSIZED TEE UNIT ECONOMICS</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Draft-only model. VAT-inclusive supplier costs are used as cash cost because current NCC context records KALM as not VAT registered. Packaging, transport, rejects, returns, ODO margin and stock are pending written confirmation. No launch or offer is authorised by this workbook.</x:v>
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Internal commercial model. The approved normal KALM retail price is R699. Supplier availability and production support are confirmed verbally by Munya. This workbook remains internal audit evidence and does not replace current OneDayOnly terms.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
-        <x:v>Recommended review configuration</x:v>
+        <x:v>Approved current configuration</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
         <x:v>KALM retail</x:v>
@@ -394,7 +415,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="14" t="str">
-        <x:v>KALM Buffalo Heavyweight Tee</x:v>
+        <x:v>KALM Signature Oversized Tee</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
         <x:v>699</x:v>
@@ -424,7 +445,28 @@
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="17" t="str">
-        <x:v>No unknown cost is set to a fictional amount. The formula outputs exclude items that are labelled PENDING QUOTE; therefore no net-margin decision is permitted from this model alone.</x:v>
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>The internal model records R85 embroidery including VAT and R0 ODO warehouse courier cost because Munya will personally deliver to Ndabeni. No internal supplier, margin or production information is customer-facing.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>